<commit_message>
update loans migration script using MongoDB
</commit_message>
<xml_diff>
--- a/models/test_data_IZ_to_IZ.xlsx
+++ b/models/test_data_IZ_to_IZ.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\projects\iz_to_iz_transfer\models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7876D6C-D77A-44BA-9D60-662AD39BD618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{441F8904-F10A-4DF5-AFDD-CF6CC1796703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="800" firstSheet="1" activeTab="4" xr2:uid="{AD365A3D-3304-46D8-98A5-452209B6D1C5}"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="12645" tabRatio="800" xr2:uid="{AD365A3D-3304-46D8-98A5-452209B6D1C5}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="156">
   <si>
     <t>Barcode</t>
   </si>
@@ -408,42 +408,15 @@
     <t>When transfering loans, make only returns in source IZ</t>
   </si>
   <si>
-    <t>If no,no loan created, but only maybe returns according to the next option</t>
-  </si>
-  <si>
     <t>Primary_id</t>
   </si>
   <si>
     <t>Barcode_s</t>
   </si>
   <si>
-    <t>MMS_id_s</t>
-  </si>
-  <si>
-    <t>Holding_id_s</t>
-  </si>
-  <si>
-    <t>Item_id_s</t>
-  </si>
-  <si>
-    <t>MMS_id_d</t>
-  </si>
-  <si>
-    <t>Holding_id_d</t>
-  </si>
-  <si>
-    <t>Item_id_d</t>
-  </si>
-  <si>
-    <t>Barcode_d</t>
-  </si>
-  <si>
     <t>Request_id_s</t>
   </si>
   <si>
-    <t>0000417644631533@test.eduid.ch</t>
-  </si>
-  <si>
     <t>UBS000034399</t>
   </si>
   <si>
@@ -453,9 +426,6 @@
     <t>A100_KUR</t>
   </si>
   <si>
-    <t>OLD_UBS000034399</t>
-  </si>
-  <si>
     <t>8.0</t>
   </si>
   <si>
@@ -541,13 +511,16 @@
   </si>
   <si>
     <t>POL-UBS-2026-214046</t>
+  </si>
+  <si>
+    <t>0000928200592230@test.eduid.ch</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -602,6 +575,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -626,13 +607,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -655,8 +637,10 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4"/>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
+    <cellStyle name="Lien hypertexte" xfId="4" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{DAFBFA39-22AE-4E9D-AC20-8AE095ED5982}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{51B8D781-AE44-4138-B03D-1D28C37B98C1}"/>
@@ -1004,7 +988,7 @@
         <v>70</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="C5" t="s">
         <v>90</v>
@@ -1043,7 +1027,7 @@
         <v>49</v>
       </c>
       <c r="C9" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:3">
@@ -1059,7 +1043,7 @@
         <v>114</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="C11" t="s">
         <v>115</v>
@@ -1070,7 +1054,7 @@
         <v>116</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="C12" t="s">
         <v>115</v>
@@ -1078,13 +1062,13 @@
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>53</v>
       </c>
       <c r="C13" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -1132,32 +1116,29 @@
         <v>113</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C19" t="s">
-        <v>120</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="1" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="B20" s="3">
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="1" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C21" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:4">
@@ -1443,10 +1424,10 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="5" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>97</v>
@@ -1712,27 +1693,27 @@
     </row>
     <row r="8" spans="1:1">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -1790,7 +1771,7 @@
         <v>62</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>
@@ -1817,17 +1798,17 @@
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="12" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="12" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="12" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -1862,16 +1843,16 @@
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -1892,47 +1873,34 @@
   <sheetPr>
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="9" width="15.7109375" customWidth="1"/>
+    <col min="1" max="2" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B1" t="s">
         <v>121</v>
       </c>
-      <c r="B1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C1" t="s">
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2" t="s">
         <v>123</v>
       </c>
-      <c r="D1" t="s">
-        <v>124</v>
-      </c>
-      <c r="E1" t="s">
-        <v>125</v>
-      </c>
-      <c r="F1" t="s">
-        <v>126</v>
-      </c>
-      <c r="G1" t="s">
-        <v>127</v>
-      </c>
-      <c r="H1" t="s">
-        <v>128</v>
-      </c>
-      <c r="I1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9">
-      <c r="A2" t="s">
-        <v>131</v>
-      </c>
-      <c r="B2" t="s">
-        <v>135</v>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B3" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1950,10 +1918,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B1" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -1975,24 +1943,24 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="5" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="5" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>52</v>
@@ -2000,10 +1968,10 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="5" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>52</v>
@@ -2011,7 +1979,7 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="5" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>53</v>

</xml_diff>